<commit_message>
fix(templates): regenerate MFRS SOCI + SOCF-Direct formulas from SSM calc linkbase
The hand-built SOCI (both variants) and SOCF-Direct templates deviated
from the calculation linkbase: orphaned OCI components, reclassification
adjustments added instead of subtracted, and inverted SOCF-Direct payment
signs. Extend regenerate_mfrs_sofp_sopl_formulas.py to cover both, pin
the regenerated formulas in tests/test_template_formulas.py, align
prompts/_sign_conventions.py + the SOCF-Direct fill workflow doc, and
snapshot the originals under backup-originals/.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XBRL-template-MFRS/Company/05-SOCI-BeforeTax.xlsx
+++ b/XBRL-template-MFRS/Company/05-SOCI-BeforeTax.xlsx
@@ -626,6 +626,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1" s="13">
       <c r="A3" s="27" t="inlineStr">
         <is>
@@ -730,8 +731,14 @@
           <t>Other comprehensive income, before tax, gains (losses) on other items</t>
         </is>
       </c>
-      <c r="B13" s="34" t="n"/>
-      <c r="C13" s="34" t="n"/>
+      <c r="B13" s="34">
+        <f>1*B11+1*B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="34">
+        <f>1*C11+1*C12</f>
+        <v/>
+      </c>
       <c r="D13" s="38" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1" s="13">
@@ -751,11 +758,11 @@
         </is>
       </c>
       <c r="B15" s="36">
-        <f>1*B11+1*B12+1*B13+1*B14</f>
+        <f>1*B13+1*B14</f>
         <v/>
       </c>
       <c r="C15" s="36">
-        <f>1*C11+1*C12+1*C13+1*C14</f>
+        <f>1*C13+1*C14</f>
         <v/>
       </c>
       <c r="D15" s="40" t="n"/>
@@ -1079,11 +1086,11 @@
         </is>
       </c>
       <c r="B43" s="36">
-        <f>1*B37-1*B40-1*B42</f>
+        <f>1*B37+-1*B40+-1*B42</f>
         <v/>
       </c>
       <c r="C43" s="36">
-        <f>1*C37-1*C40-1*C42</f>
+        <f>1*C37+-1*C40+-1*C42</f>
         <v/>
       </c>
       <c r="D43" s="40" t="n"/>

</xml_diff>